<commit_message>
Add Env Var Name column to API requirements sheet and .env.example
Maps each API/sandbox in the requirements list to the environment
variable name the app will read, and adds zkd-app/.env.example so
keys obtained from the linked signup pages can be dropped straight
into a .env.local.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ByBjKAHCipoHKj626oq4k7
</commit_message>
<xml_diff>
--- a/round2-api-requirements.xlsx
+++ b/round2-api-requirements.xlsx
@@ -10,7 +10,7 @@
     <sheet name="API Requirements" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Requirements'!$A$1:$I$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'API Requirements'!$A$1:$J$19</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,6 +31,14 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="6">
@@ -91,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -102,7 +110,13 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -473,17 +487,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -527,6 +542,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Env Var Name</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -569,6 +589,11 @@
           <t>Primary choice if Amex grants access in time</t>
         </is>
       </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>AMEX_VPAY_API_KEY, AMEX_VPAY_API_SECRET</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -591,7 +616,7 @@
           <t>Lets you demo the same payment safety guarantee without waiting on an Amex partnership</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -601,7 +626,7 @@
           <t>Test mode is free with unlimited fake test cards</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" s="6" t="inlineStr">
         <is>
           <t>https://stripe.com/issuing</t>
         </is>
@@ -609,6 +634,11 @@
       <c r="H3" s="2" t="inlineStr">
         <is>
           <t>Recommended fallback if Amex sandbox isn't available in time</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>STRIPE_SECRET_KEY</t>
         </is>
       </c>
     </row>
@@ -633,7 +663,7 @@
           <t>Weather is the single largest driver of Indian domestic cancellations</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -643,7 +673,7 @@
           <t>Fully free public API, no key, no signup</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>https://aviationweather.gov/data/api/</t>
         </is>
@@ -651,6 +681,11 @@
       <c r="H4" s="2" t="inlineStr">
         <is>
           <t>Best primary source - use this one first</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>No key required — public API</t>
         </is>
       </c>
     </row>
@@ -675,7 +710,7 @@
           <t>Free fallback if the NOAA endpoint is unavailable</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -685,7 +720,7 @@
           <t>Free for non-commercial use, up to 10000 calls/day, no key</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>https://open-meteo.com/</t>
         </is>
@@ -695,9 +730,14 @@
           <t>Not aviation-grade (no visibility/crosswind) - backup only</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> not primary</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>No key required — public API</t>
         </is>
       </c>
     </row>
@@ -722,7 +762,7 @@
           <t>Localizes the weather signal to Indian airports specifically</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -732,7 +772,7 @@
           <t>Free but needs registration/MoU</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>https://mausam.imd.gov.in/</t>
         </is>
@@ -740,6 +780,11 @@
       <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Ask mentor if IIT Madras has institutional access</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>IMD_API_KEY</t>
         </is>
       </c>
     </row>
@@ -764,7 +809,7 @@
           <t>This is the most important feed in the whole system - no trigger without it</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Yes (limited)</t>
         </is>
@@ -774,7 +819,7 @@
           <t>100 requests/month free, 1 req per 60s rate limit on free tier</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>https://aviationstack.com/</t>
         </is>
@@ -784,9 +829,14 @@
           <t>Already sandboxed per your docs - verify the key still works; too limited for live polling at scale</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> fine for a scripted demo</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>AVIATIONSTACK_API_KEY</t>
         </is>
       </c>
     </row>
@@ -811,7 +861,7 @@
           <t>Free real-time aircraft position feed for the aircraft-rotation risk feature</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -821,7 +871,7 @@
           <t>Anonymous: 400 requests per 2.2 hours; registered account: ~8000 credits/day</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
         <is>
           <t>https://opensky-network.org/</t>
         </is>
@@ -829,6 +879,11 @@
       <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Good free source specifically for the rotation feature</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>OPENSKY_CLIENT_ID, OPENSKY_CLIENT_SECRET</t>
         </is>
       </c>
     </row>
@@ -853,7 +908,7 @@
           <t>Best tail-number-linked rotation data - the 2nd heaviest risk feature (~26%)</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>Yes (small)</t>
         </is>
@@ -863,7 +918,7 @@
           <t>Personal tier: about $5 of free monthly query usage, personal/academic use only</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>https://www.flightaware.com/commercial/aeroapi/</t>
         </is>
@@ -873,9 +928,14 @@
           <t>Enough for demo-scale queries</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> not production volume</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>FLIGHTAWARE_API_KEY</t>
         </is>
       </c>
     </row>
@@ -920,9 +980,14 @@
           <t>https://www.cirium.com/</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Ask mentor if Amex can broker hackathon access</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>CIRIUM_API_KEY</t>
         </is>
       </c>
     </row>
@@ -947,7 +1012,7 @@
           <t>Sets the prior risk baseline independent of today's weather/rotation</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -957,7 +1022,7 @@
           <t>Free, published; a community-scraped CSV dataset already exists on GitHub</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>https://github.com/Vonter/india-aviation-traffic</t>
         </is>
@@ -965,6 +1030,11 @@
       <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Much faster than scraping dgca.gov.in yourself</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>No key — static dataset URL</t>
         </is>
       </c>
     </row>
@@ -989,7 +1059,7 @@
           <t>Makes the rollback/compensation demo real instead of narrated</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -999,7 +1069,7 @@
           <t>Free sandbox, unlimited test balance; Duffel even publishes a hackathon starter kit</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>https://duffel.com/</t>
         </is>
@@ -1007,6 +1077,11 @@
       <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Use the Duffel Airways sandbox airline (LHR-JFK) for reliability</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>DUFFEL_ACCESS_TOKEN</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1106,7 @@
           <t>Wider domestic-carrier coverage than Duffel alone</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Yes (sandbox only)</t>
         </is>
@@ -1041,7 +1116,7 @@
           <t>Free self-serve sandbox; production access requires a paid agreement</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>https://developer.sabre.com/</t>
         </is>
@@ -1049,6 +1124,11 @@
       <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Good for the demo; not usable for real production booking</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>SABRE_CLIENT_ID, SABRE_CLIENT_SECRET</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1153,7 @@
           <t>Needed for the duty-of-care hotel leg (Outcome C - next-day recovery)</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1083,7 +1163,7 @@
           <t>Free sandbox, no credit card required; test card 4242 4242 4242 4242</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>https://liteapi.travel/</t>
         </is>
@@ -1091,6 +1171,11 @@
       <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Already sandboxed per your docs - verify the key still works</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>LITEAPI_API_KEY</t>
         </is>
       </c>
     </row>
@@ -1135,6 +1220,11 @@
           <t>Recommend keeping this mocked and stating that plainly to judges</t>
         </is>
       </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>UBER_API_KEY</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1157,7 +1247,7 @@
           <t>This is the biggest gap today - zero LLM calls exist anywhere in the repo, despite it being the headline architecture claim</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="7" t="inlineStr">
         <is>
           <t>Yes (small)</t>
         </is>
@@ -1167,7 +1257,7 @@
           <t>New accounts get a small trial credit (roughly $5); academic/research applicants can get up to $20000 over 6 months; occasional hackathon-specific credit programs</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>https://console.anthropic.com/</t>
         </is>
@@ -1175,6 +1265,11 @@
       <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Ask the mentor whether Amex/Anthropic is running a credit program for this hackathon</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
+        <is>
+          <t>ANTHROPIC_API_KEY</t>
         </is>
       </c>
     </row>
@@ -1199,7 +1294,7 @@
           <t>Fallback / comparison to the Anthropic option</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Yes (small)</t>
         </is>
@@ -1209,7 +1304,7 @@
           <t>New accounts get a limited free trial credit (varies)</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>https://platform.openai.com/</t>
         </is>
@@ -1217,6 +1312,11 @@
       <c r="H17" s="2" t="inlineStr">
         <is>
           <t>Use whichever provider has usable credits first</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>OPENAI_API_KEY</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1341,7 @@
           <t>Compliance grounding already cited in your docs - keep the reference current</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1251,7 +1351,7 @@
           <t>Public law text</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>https://www.meity.gov.in/</t>
         </is>
@@ -1261,9 +1361,14 @@
           <t>No API - just the reference document</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve"> no build cost</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Reference doc only, not an API</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1393,7 @@
           <t>Currently carries the unverified `deck` evidence tier in your docs - needs a primary-source re-check</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
@@ -1298,7 +1403,7 @@
           <t>Public regulation text</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>https://www.dgca.gov.in/</t>
         </is>
@@ -1308,9 +1413,31 @@
           <t>Your own docs already flag this as outstanding - re-retrieve before final submission</t>
         </is>
       </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Reference doc only, not an API</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I19"/>
+  <autoFilter ref="A1:J19"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId15"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>